<commit_message>
Added Playwright and updated consistency throughout the scenarios
</commit_message>
<xml_diff>
--- a/docs/asset-management/PromptCraft_Voice_Recording_Tracker.xlsx
+++ b/docs/asset-management/PromptCraft_Voice_Recording_Tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R9d4db76357b8496b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recording Queue" sheetId="2" r:id="R3f4900b60a77459f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Needs Decision" sheetId="3" r:id="R19c3d7b9a01b472e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retired - Do Not Record" sheetId="4" r:id="Raab6f61e738d4c8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R192d2ed5b8064b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recording Queue" sheetId="2" r:id="R5bbf0d93c64249d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Needs Decision" sheetId="3" r:id="R3656174da7144179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retired - Do Not Record" sheetId="4" r:id="Rea71be5962384e1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -492,7 +492,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="8" t="str">
-        <x:v>Verified against the active V429 dialogue source · dialogue asset 149 · Phase 6 / patch 527 · current roadmap labels with legacy recording filenames preserved</x:v>
+        <x:v>Verified against active V429 dialogue source · dialogue asset 149 · Dialogue draft through patch 534 · legacy recording filenames preserved</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" customHeight="1">
@@ -513,13 +513,11 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="15" customHeight="1">
-      <x:c r="A5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Ready lines</x:t>
-        </x:is>
+      <x:c r="A5" t="str">
+        <x:v>Ready lines</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:v>68</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D5" s="2" t="inlineStr">
         <x:is>
@@ -533,13 +531,11 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="15" customHeight="1">
-      <x:c r="A6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Professor Pixel</x:t>
-        </x:is>
+      <x:c r="A6" t="str">
+        <x:v>Professor Pixel ready lines</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>43</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D6" s="2" t="inlineStr">
         <x:is>
@@ -553,13 +549,11 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="15" customHeight="1">
-      <x:c r="A7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Jordan</x:t>
-        </x:is>
+      <x:c r="A7" t="str">
+        <x:v>Jordan ready lines</x:v>
       </x:c>
       <x:c r="B7" t="n">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="2" t="inlineStr">
         <x:is>
@@ -573,10 +567,8 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="15" customHeight="1">
-      <x:c r="A8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Commercial-model names</x:t>
-        </x:is>
+      <x:c r="A8" t="str">
+        <x:v>Commercial-model names</x:v>
       </x:c>
       <x:c r="B8" t="n">
         <x:v>0</x:v>
@@ -593,10 +585,8 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="15" customHeight="1">
-      <x:c r="A9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Eli</x:t>
-        </x:is>
+      <x:c r="A9" t="str">
+        <x:v>Eli ready lines</x:v>
       </x:c>
       <x:c r="B9" t="n">
         <x:v>18</x:v>
@@ -604,7 +594,14 @@
       <x:c r="D9" s="2" t="n"/>
       <x:c r="E9" s="10" t="n"/>
     </x:row>
-    <x:row r="10" ht="15" customHeight="1"/>
+    <x:row r="10" ht="15" customHeight="1">
+      <x:c r="A10" t="str">
+        <x:v>Scenario 3 draft lines</x:v>
+      </x:c>
+      <x:c r="B10" t="n">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
     <x:row r="11">
       <x:c r="A11" s="11" t="inlineStr">
         <x:is>
@@ -614,7 +611,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="12" t="str">
-        <x:v>Retired the old S1: Engagement queue and retained it only on the retired sheet. The active queue contains 43 Professor Pixel lines, 18 Eli lines for S1: The Content Avalanche, and 7 Jordan lines for S3: The Confident Student Problem. Scenario-02 and s2 filename tokens remain only for source and saved-data compatibility. Current S2: Access Is Part of the Design is still a development shell and has no recording queue.</x:v>
+        <x:v>The active queue contains 54 lines that are ready to record and 14 revised Scenario 3 lines marked Draft, Do Not Record. Scenario 3 now references the planned Week 4 Canvas module, 84% quiz result, practice check, feedback, and reflection activity. Scenario-02 and s2 filename tokens remain only for source and saved-data compatibility. Current S2: Access Is Part of the Design remains a development shell and has no recording queue.</x:v>
       </x:c>
     </x:row>
     <x:row r="13"/>
@@ -2450,7 +2447,7 @@
         <x:v>neutral</x:v>
       </x:c>
       <x:c r="F56" s="5" t="str">
-        <x:v>Meet Jordan. He completes his assignments, earns passing grades, and seems to be doing fine.</x:v>
+        <x:v>Meet Jordan. He finished the Week 4 Canvas module and earned 84% on the module quiz. From the gradebook, everything looks fine.</x:v>
       </x:c>
       <x:c r="G56" s="5" t="str">
         <x:v>p86.mp3</x:v>
@@ -2459,7 +2456,7 @@
         <x:v>assets/audio/voice/professor-pixel/scenario-02/p86.mp3</x:v>
       </x:c>
       <x:c r="I56" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J56" s="5" t="str">
         <x:v>High</x:v>
@@ -2482,7 +2479,7 @@
         <x:v>thinking</x:v>
       </x:c>
       <x:c r="F57" s="5" t="str">
-        <x:v>His performance improved. His strategy might have worked. But listen carefully to what Jordan actually knows about his learning.</x:v>
+        <x:v>The module shows what Jordan opened and what he scored. It does not show which strategy changed his understanding or where that understanding still breaks down.</x:v>
       </x:c>
       <x:c r="G57" s="5" t="str">
         <x:v>p88.mp3</x:v>
@@ -2491,7 +2488,7 @@
         <x:v>assets/audio/voice/professor-pixel/scenario-02/p88.mp3</x:v>
       </x:c>
       <x:c r="I57" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J57" s="5" t="str">
         <x:v>High</x:v>
@@ -2514,7 +2511,7 @@
         <x:v>encouraging</x:v>
       </x:c>
       <x:c r="F58" s="5" t="str">
-        <x:v>Let's figure out what's missing.</x:v>
+        <x:v>Inspect the Canvas path and find the missing link between Jordan's strategy, the quiz result, and his next decision.</x:v>
       </x:c>
       <x:c r="G58" s="5" t="str">
         <x:v>p89.mp3</x:v>
@@ -2523,7 +2520,7 @@
         <x:v>assets/audio/voice/professor-pixel/scenario-02/p89.mp3</x:v>
       </x:c>
       <x:c r="I58" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J58" s="5" t="str">
         <x:v>High</x:v>
@@ -2546,7 +2543,7 @@
         <x:v>proud</x:v>
       </x:c>
       <x:c r="F59" s="5" t="str">
-        <x:v>That's the hidden problem. Jordan has an outcome and a strategy, but no evidence connecting the two. He cannot judge what helped or use that judgment to make his next decision.</x:v>
+        <x:v>That's the hidden problem. Canvas shows Jordan's module activity and grade, but not evidence connecting his study strategy to what he actually understood. He cannot make an informed next decision yet.</x:v>
       </x:c>
       <x:c r="G59" s="5" t="str">
         <x:v>p90.mp3</x:v>
@@ -2555,7 +2552,7 @@
         <x:v>assets/audio/voice/professor-pixel/scenario-02/p90.mp3</x:v>
       </x:c>
       <x:c r="I59" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J59" s="5" t="str">
         <x:v>High</x:v>
@@ -2578,7 +2575,7 @@
         <x:v>thinking</x:v>
       </x:c>
       <x:c r="F60" s="5" t="str">
-        <x:v>Rereading may not be his best strategy, but replacing it does not solve the deeper problem. Jordan still needs a way to tell why a strategy worked or failed.</x:v>
+        <x:v>Rereading may not be his best strategy, but replacing it inside the next Canvas module does not solve the deeper problem. Jordan still needs evidence showing why a strategy worked or failed.</x:v>
       </x:c>
       <x:c r="G60" s="5" t="str">
         <x:v>p91.mp3</x:v>
@@ -2587,7 +2584,7 @@
         <x:v>assets/audio/voice/professor-pixel/scenario-02/p91.mp3</x:v>
       </x:c>
       <x:c r="I60" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J60" s="5" t="str">
         <x:v>High</x:v>
@@ -2610,7 +2607,7 @@
         <x:v>skeptical</x:v>
       </x:c>
       <x:c r="F61" s="5" t="str">
-        <x:v>Jordan completed the work and is trying to understand the result. The evidence points somewhere other than motivation.</x:v>
+        <x:v>Jordan completed the Canvas module and is trying to understand the result. The evidence points to a missing learning check, not a motivation problem.</x:v>
       </x:c>
       <x:c r="G61" s="5" t="str">
         <x:v>p92.mp3</x:v>
@@ -2619,7 +2616,7 @@
         <x:v>assets/audio/voice/professor-pixel/scenario-02/p92.mp3</x:v>
       </x:c>
       <x:c r="I61" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J61" s="5" t="str">
         <x:v>High</x:v>
@@ -2642,7 +2639,7 @@
         <x:v>neutral</x:v>
       </x:c>
       <x:c r="F62" s="5" t="str">
-        <x:v>The grade tells us how Jordan performed. It does not tell Jordan what produced the learning or what he should do next.</x:v>
+        <x:v>The Canvas grade already tells us how Jordan performed. A higher score still does not tell him what produced the learning or what he should do next.</x:v>
       </x:c>
       <x:c r="G62" s="5" t="str">
         <x:v>p93.mp3</x:v>
@@ -2651,7 +2648,7 @@
         <x:v>assets/audio/voice/professor-pixel/scenario-02/p93.mp3</x:v>
       </x:c>
       <x:c r="I62" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J62" s="5" t="str">
         <x:v>High</x:v>
@@ -2674,7 +2671,7 @@
         <x:v>neutral</x:v>
       </x:c>
       <x:c r="F63" s="5" t="str">
-        <x:v>I got an 84 on this assignment. That's better than last time, so I guess something worked.</x:v>
+        <x:v>Canvas shows my score improved, but I don't know why. I got an 84% on the module quiz after getting 76% last time.</x:v>
       </x:c>
       <x:c r="G63" s="5" t="str">
         <x:v>jordan-s2-01.mp3</x:v>
@@ -2683,7 +2680,7 @@
         <x:v>assets/audio/voice/students/jordan/scenario-02/jordan-s2-01.mp3</x:v>
       </x:c>
       <x:c r="I63" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J63" s="5" t="str">
         <x:v>High</x:v>
@@ -2706,7 +2703,7 @@
         <x:v>uncertain</x:v>
       </x:c>
       <x:c r="F64" s="5" t="str">
-        <x:v>I reread the chapter a few times. Some parts eventually made more sense, but I couldn't tell you what actually helped.</x:v>
+        <x:v>I reread the module page three times before the quiz. Some parts felt familiar, but I still couldn't explain the difference between the two concepts without my notes.</x:v>
       </x:c>
       <x:c r="G64" s="5" t="str">
         <x:v>jordan-s2-02.mp3</x:v>
@@ -2715,7 +2712,7 @@
         <x:v>assets/audio/voice/students/jordan/scenario-02/jordan-s2-02.mp3</x:v>
       </x:c>
       <x:c r="I64" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J64" s="5" t="str">
         <x:v>High</x:v>
@@ -2738,7 +2735,7 @@
         <x:v>frustrated</x:v>
       </x:c>
       <x:c r="F65" s="5" t="str">
-        <x:v>Next time I'll probably reread everything again and hope it works.</x:v>
+        <x:v>The next module opens Monday. I'll probably reread everything again and hope the score keeps improving.</x:v>
       </x:c>
       <x:c r="G65" s="5" t="str">
         <x:v>jordan-s2-03.mp3</x:v>
@@ -2747,7 +2744,7 @@
         <x:v>assets/audio/voice/students/jordan/scenario-02/jordan-s2-03.mp3</x:v>
       </x:c>
       <x:c r="I65" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J65" s="5" t="str">
         <x:v>High</x:v>
@@ -2770,7 +2767,7 @@
         <x:v>confident</x:v>
       </x:c>
       <x:c r="F66" s="5" t="str">
-        <x:v>I’d say I’m a four out of five. I feel better about it this time.</x:v>
+        <x:v>In the Canvas reflection, I’d rate my confidence four out of five. I feel better, but I still can't explain what the rereading changed.</x:v>
       </x:c>
       <x:c r="G66" s="5" t="str">
         <x:v>jordan-s2-intervention-confidence.mp3</x:v>
@@ -2779,7 +2776,7 @@
         <x:v>assets/audio/voice/students/jordan/scenario-02/jordan-s2-intervention-confidence.mp3</x:v>
       </x:c>
       <x:c r="I66" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J66" s="5" t="str">
         <x:v>High</x:v>
@@ -2802,7 +2799,7 @@
         <x:v>thinking</x:v>
       </x:c>
       <x:c r="F67" s="5" t="str">
-        <x:v>I reread the chapter three times and highlighted the parts that seemed important.</x:v>
+        <x:v>I reread the module page three times and highlighted the parts that seemed important.</x:v>
       </x:c>
       <x:c r="G67" s="5" t="str">
         <x:v>jordan-s2-intervention-strategy.mp3</x:v>
@@ -2811,7 +2808,7 @@
         <x:v>assets/audio/voice/students/jordan/scenario-02/jordan-s2-intervention-strategy.mp3</x:v>
       </x:c>
       <x:c r="I67" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J67" s="5" t="str">
         <x:v>High</x:v>
@@ -2834,7 +2831,7 @@
         <x:v>confident</x:v>
       </x:c>
       <x:c r="F68" s="5" t="str">
-        <x:v>I got an 84 instead of a 76, so rereading must have worked.</x:v>
+        <x:v>My Canvas grade went from 76% to 84%, so rereading must have worked.</x:v>
       </x:c>
       <x:c r="G68" s="5" t="str">
         <x:v>jordan-s2-intervention-grade.mp3</x:v>
@@ -2843,7 +2840,7 @@
         <x:v>assets/audio/voice/students/jordan/scenario-02/jordan-s2-intervention-grade.mp3</x:v>
       </x:c>
       <x:c r="I68" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J68" s="5" t="str">
         <x:v>High</x:v>
@@ -2866,7 +2863,7 @@
         <x:v>thinking</x:v>
       </x:c>
       <x:c r="F69" s="5" t="str">
-        <x:v>I could define both concepts, but without my notes I still couldn’t explain the difference. Rereading helped me recognize them, but it didn’t help me compare them. I need to try examples next.</x:v>
+        <x:v>On the Canvas practice check, I could define both concepts, but without my notes I still couldn’t explain the difference. Rereading helped me recognize them, but it didn’t help me compare them. I need to try examples next.</x:v>
       </x:c>
       <x:c r="G69" s="5" t="str">
         <x:v>jordan-s2-intervention-evidence.mp3</x:v>
@@ -2875,7 +2872,7 @@
         <x:v>assets/audio/voice/students/jordan/scenario-02/jordan-s2-intervention-evidence.mp3</x:v>
       </x:c>
       <x:c r="I69" s="5" t="str">
-        <x:v>Ready to Record</x:v>
+        <x:v>Draft, Do Not Record</x:v>
       </x:c>
       <x:c r="J69" s="5" t="str">
         <x:v>High</x:v>
@@ -2889,7 +2886,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb07dfc2224a54914"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dd1a4efc35e4c2a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3064,7 +3061,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1ddbb4b171c4ec6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cce150aefae4896"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3272,7 +3269,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0f07bfe831a4169"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf5c945c3c4d4938"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>